<commit_message>
Add tariffs, CO2 offset, seasonal battery DoD, sizing limits, peak-demand inverter, full-year load; fix Streamlit circular import
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/microgrid_inputs.xlsx
+++ b/microgrid_inputs.xlsx
@@ -12,8 +12,9 @@
     <sheet name="batteries" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="inverters" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="diesel_generators" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="bos" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="load" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="tariff" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="bos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="load" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -486,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -501,7 +502,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -591,74 +591,76 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>tariff</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>match a row in 'tariff'; blank = flat grid_price</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>PROJECT</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Parameter</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>lifetime</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>years</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>grid_capacity_kW</t>
+          <t>lifetime</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>10000</v>
+        <v>20</v>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>kW connection limit</t>
+          <t>years</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>grid_price</t>
+          <t>grid_capacity_kW</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>0.15</v>
+        <v>10000</v>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>$/kWh</t>
+          <t>kW connection limit</t>
         </is>
       </c>
     </row>
@@ -729,7 +731,7 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
@@ -759,7 +761,7 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
@@ -783,102 +785,132 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr"/>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>battery_dod_jan</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>min SoC floor for months Oct-Mar (0.2 = use 80%)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>battery_dod_jul</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>min SoC floor for months Apr-Sep (0.5 = use 50%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>FUEL &amp; TANK  (the diesel model is chosen above from 'diesel_generators')</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Parameter</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>tank_min_kWh</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>kWh</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>tank_max_kWh</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="n">
-        <v>5000</v>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>kWh</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>tank_dod</t>
+          <t>tank_min_kWh</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>kWh</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>fuel_usd_per_L</t>
+          <t>tank_max_kWh</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>1.5</v>
+        <v>5000</v>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>$/L (converts to $/kWh using fixed diesel density)</t>
+          <t>kWh</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
+          <t>tank_dod</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>fuel_usd_per_L</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>$/L (converts to $/kWh using fixed diesel density)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
           <t>fuel_kWh_per_kg</t>
         </is>
       </c>
-      <c r="B30" s="5" t="n">
+      <c r="B32" s="5" t="n">
         <v>11.9</v>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>kWh/kg (informational; price is $/L)</t>
         </is>
@@ -887,13 +919,13 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A11:C11"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A9:C9"/>
     <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A26:C26"/>
   </mergeCells>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=solar_panels!$A$2:$A$100</formula1>
     </dataValidation>
@@ -905,6 +937,9 @@
     </dataValidation>
     <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=diesel_generators!$A$2:$A$100</formula1>
+    </dataValidation>
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=tariff!$A$2:$A$100</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1412,6 +1447,148 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>block_kWh</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>block_rate_TZS</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>energy_TZS_per_kWh</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>service_TZS_per_month</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>demand_TZS_per_kWp_month</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>350</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="8" t="n">
+        <v>292</v>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>195</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>14233</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>T3-MV</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>157</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>16769</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>13200</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1684,7 +1861,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add grid outage hours (grid_cut_hours) with robust mixed-format parsing
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/microgrid_inputs.xlsx
+++ b/microgrid_inputs.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -682,97 +682,95 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>lat</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>-3.314732</v>
-      </c>
+          <t>grid_cut_hours</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr"/>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>PVGIS site latitude (decimal degrees)</t>
+          <t>force grid import = 0, e.g. '3000-3003' or '100,200'</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>lon</t>
+          <t>lat</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>37.326358</v>
+        <v>-3.314732</v>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>PVGIS site longitude (decimal degrees)</t>
+          <t>PVGIS site latitude (decimal degrees)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>solar_max_kW</t>
+          <t>lon</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>100000</v>
+        <v>37.326358</v>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>upper bound for solar sizing (kW)</t>
+          <t>PVGIS site longitude (decimal degrees)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>solar_min_kW</t>
+          <t>solar_max_kW</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>lower bound — force at least this much solar (kW)</t>
+          <t>upper bound for solar sizing (kW)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>battery_max_kWh</t>
+          <t>solar_min_kW</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>upper bound for battery sizing (kWh)</t>
+          <t>lower bound — force at least this much solar (kW)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>battery_min_kWh</t>
+          <t>battery_max_kWh</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>lower bound — force at least this much battery (kWh)</t>
+          <t>upper bound for battery sizing (kWh)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>diesel_min_kW</t>
+          <t>battery_min_kWh</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
@@ -780,29 +778,29 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>lower bound — force at least this much diesel (kW)</t>
+          <t>lower bound — force at least this much battery (kWh)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>battery_dod_jan</t>
+          <t>diesel_min_kW</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>min SoC floor for months Oct-Mar (0.2 = use 80%)</t>
+          <t>lower bound — force at least this much diesel (kW)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>battery_dod_jul</t>
+          <t>battery_dod_jan</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
@@ -810,60 +808,60 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
+          <t>min SoC floor for months Oct-Mar (0.2 = use 80%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>battery_dod_jul</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
           <t>min SoC floor for months Apr-Sep (0.5 = use 50%)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
-    </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>FUEL &amp; TANK  (the diesel model is chosen above from 'diesel_generators')</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Parameter</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>tank_min_kWh</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>kWh</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>tank_max_kWh</t>
+          <t>tank_min_kWh</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
@@ -874,43 +872,58 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>tank_dod</t>
+          <t>tank_max_kWh</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>0.1</v>
+        <v>5000</v>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>kWh</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>fuel_usd_per_L</t>
+          <t>tank_dod</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>1.5</v>
+        <v>0.1</v>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>$/L (converts to $/kWh using fixed diesel density)</t>
+          <t>0-1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
+          <t>fuel_usd_per_L</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>$/L (converts to $/kWh using fixed diesel density)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
           <t>fuel_kWh_per_kg</t>
         </is>
       </c>
-      <c r="B32" s="5" t="n">
+      <c r="B33" s="5" t="n">
         <v>11.9</v>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>kWh/kg (informational; price is $/L)</t>
         </is>
@@ -919,9 +932,9 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A25:C25"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A27:C27"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A26:C26"/>
   </mergeCells>

</xml_diff>